<commit_message>
updated: readme and xlsx
</commit_message>
<xml_diff>
--- a/Results.xlsx
+++ b/Results.xlsx
@@ -8,10 +8,10 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Counts" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Counts_2" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="Details" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="Sheet4" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="counts_skills" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="counts_comp_skills" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="skills_coded_detail" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="media_education" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -908,6 +908,7 @@
     </font>
     <font>
       <sz val="10"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -1111,7 +1112,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Counts_2!$C$1</c:f>
+              <c:f>counts_comp_skills!$C$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1136,11 +1137,15 @@
               <a:p>
                 <a:pPr>
                   <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:latin typeface="Arial"/>
                   </a:defRPr>
                 </a:pPr>
               </a:p>
             </c:txPr>
+            <c:dLblPos val="ctr"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="0"/>
             <c:showCatName val="0"/>
@@ -1156,7 +1161,7 @@
           </c:dLbls>
           <c:cat>
             <c:multiLvlStrRef>
-              <c:f>Counts_2!$A$2:$B$13</c:f>
+              <c:f>counts_comp_skills!$A$2:$B$13</c:f>
               <c:multiLvlStrCache>
                 <c:ptCount val="12"/>
                 <c:lvl>
@@ -1219,7 +1224,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Counts_2!$C$2:$C$13</c:f>
+              <c:f>counts_comp_skills!$C$2:$C$13</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="12"/>
@@ -1268,7 +1273,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>Counts_2!$D$1</c:f>
+              <c:f>counts_comp_skills!$D$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1293,11 +1298,15 @@
               <a:p>
                 <a:pPr>
                   <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:latin typeface="Arial"/>
                   </a:defRPr>
                 </a:pPr>
               </a:p>
             </c:txPr>
+            <c:dLblPos val="ctr"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="0"/>
             <c:showCatName val="0"/>
@@ -1313,7 +1322,7 @@
           </c:dLbls>
           <c:cat>
             <c:multiLvlStrRef>
-              <c:f>Counts_2!$A$2:$B$13</c:f>
+              <c:f>counts_comp_skills!$A$2:$B$13</c:f>
               <c:multiLvlStrCache>
                 <c:ptCount val="12"/>
                 <c:lvl>
@@ -1376,7 +1385,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Counts_2!$D$2:$D$13</c:f>
+              <c:f>counts_comp_skills!$D$2:$D$13</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="12"/>
@@ -1425,7 +1434,7 @@
           <c:order val="2"/>
           <c:tx>
             <c:strRef>
-              <c:f>Counts_2!$E$1</c:f>
+              <c:f>counts_comp_skills!$E$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1450,11 +1459,15 @@
               <a:p>
                 <a:pPr>
                   <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:latin typeface="Arial"/>
                   </a:defRPr>
                 </a:pPr>
               </a:p>
             </c:txPr>
+            <c:dLblPos val="ctr"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="0"/>
             <c:showCatName val="0"/>
@@ -1470,7 +1483,7 @@
           </c:dLbls>
           <c:cat>
             <c:multiLvlStrRef>
-              <c:f>Counts_2!$A$2:$B$13</c:f>
+              <c:f>counts_comp_skills!$A$2:$B$13</c:f>
               <c:multiLvlStrCache>
                 <c:ptCount val="12"/>
                 <c:lvl>
@@ -1533,7 +1546,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Counts_2!$E$2:$E$13</c:f>
+              <c:f>counts_comp_skills!$E$2:$E$13</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="12"/>
@@ -1582,7 +1595,7 @@
           <c:order val="3"/>
           <c:tx>
             <c:strRef>
-              <c:f>Counts_2!$F$1</c:f>
+              <c:f>counts_comp_skills!$F$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1607,11 +1620,15 @@
               <a:p>
                 <a:pPr>
                   <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:latin typeface="Arial"/>
                   </a:defRPr>
                 </a:pPr>
               </a:p>
             </c:txPr>
+            <c:dLblPos val="ctr"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="0"/>
             <c:showCatName val="0"/>
@@ -1627,7 +1644,7 @@
           </c:dLbls>
           <c:cat>
             <c:multiLvlStrRef>
-              <c:f>Counts_2!$A$2:$B$13</c:f>
+              <c:f>counts_comp_skills!$A$2:$B$13</c:f>
               <c:multiLvlStrCache>
                 <c:ptCount val="12"/>
                 <c:lvl>
@@ -1690,7 +1707,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Counts_2!$F$2:$F$13</c:f>
+              <c:f>counts_comp_skills!$F$2:$F$13</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="12"/>
@@ -1739,7 +1756,7 @@
           <c:order val="4"/>
           <c:tx>
             <c:strRef>
-              <c:f>Counts_2!$G$1</c:f>
+              <c:f>counts_comp_skills!$G$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1764,11 +1781,15 @@
               <a:p>
                 <a:pPr>
                   <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:latin typeface="Arial"/>
                   </a:defRPr>
                 </a:pPr>
               </a:p>
             </c:txPr>
+            <c:dLblPos val="ctr"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="0"/>
             <c:showCatName val="0"/>
@@ -1784,7 +1805,7 @@
           </c:dLbls>
           <c:cat>
             <c:multiLvlStrRef>
-              <c:f>Counts_2!$A$2:$B$13</c:f>
+              <c:f>counts_comp_skills!$A$2:$B$13</c:f>
               <c:multiLvlStrCache>
                 <c:ptCount val="12"/>
                 <c:lvl>
@@ -1847,7 +1868,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Counts_2!$G$2:$G$13</c:f>
+              <c:f>counts_comp_skills!$G$2:$G$13</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="12"/>
@@ -1896,7 +1917,7 @@
           <c:order val="5"/>
           <c:tx>
             <c:strRef>
-              <c:f>Counts_2!$H$1</c:f>
+              <c:f>counts_comp_skills!$H$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1921,11 +1942,15 @@
               <a:p>
                 <a:pPr>
                   <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:latin typeface="Arial"/>
                   </a:defRPr>
                 </a:pPr>
               </a:p>
             </c:txPr>
+            <c:dLblPos val="ctr"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="0"/>
             <c:showCatName val="0"/>
@@ -1941,7 +1966,7 @@
           </c:dLbls>
           <c:cat>
             <c:multiLvlStrRef>
-              <c:f>Counts_2!$A$2:$B$13</c:f>
+              <c:f>counts_comp_skills!$A$2:$B$13</c:f>
               <c:multiLvlStrCache>
                 <c:ptCount val="12"/>
                 <c:lvl>
@@ -2004,7 +2029,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Counts_2!$H$2:$H$13</c:f>
+              <c:f>counts_comp_skills!$H$2:$H$13</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="12"/>
@@ -2053,7 +2078,7 @@
           <c:order val="6"/>
           <c:tx>
             <c:strRef>
-              <c:f>Counts_2!$I$1</c:f>
+              <c:f>counts_comp_skills!$I$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -2078,11 +2103,15 @@
               <a:p>
                 <a:pPr>
                   <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:latin typeface="Arial"/>
                   </a:defRPr>
                 </a:pPr>
               </a:p>
             </c:txPr>
+            <c:dLblPos val="ctr"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="0"/>
             <c:showCatName val="0"/>
@@ -2098,7 +2127,7 @@
           </c:dLbls>
           <c:cat>
             <c:multiLvlStrRef>
-              <c:f>Counts_2!$A$2:$B$13</c:f>
+              <c:f>counts_comp_skills!$A$2:$B$13</c:f>
               <c:multiLvlStrCache>
                 <c:ptCount val="12"/>
                 <c:lvl>
@@ -2161,7 +2190,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Counts_2!$I$2:$I$13</c:f>
+              <c:f>counts_comp_skills!$I$2:$I$13</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="12"/>
@@ -2207,17 +2236,17 @@
         </c:ser>
         <c:gapWidth val="100"/>
         <c:overlap val="100"/>
-        <c:axId val="61456343"/>
-        <c:axId val="21032889"/>
+        <c:axId val="89368574"/>
+        <c:axId val="37443596"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="61456343"/>
+        <c:axId val="89368574"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="General" sourceLinked="0"/>
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -2234,12 +2263,15 @@
           <a:p>
             <a:pPr>
               <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
                 <a:latin typeface="Arial"/>
               </a:defRPr>
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="21032889"/>
+        <c:crossAx val="37443596"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2247,7 +2279,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="21032889"/>
+        <c:axId val="37443596"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2262,7 +2294,7 @@
             </a:ln>
           </c:spPr>
         </c:majorGridlines>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="General" sourceLinked="0"/>
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -2279,12 +2311,15 @@
           <a:p>
             <a:pPr>
               <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
                 <a:latin typeface="Arial"/>
               </a:defRPr>
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="61456343"/>
+        <c:crossAx val="89368574"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2312,6 +2347,9 @@
         <a:p>
           <a:pPr>
             <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
               <a:latin typeface="Arial"/>
             </a:defRPr>
           </a:pPr>
@@ -2343,9 +2381,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>1253160</xdr:colOff>
+      <xdr:colOff>1252800</xdr:colOff>
       <xdr:row>33</xdr:row>
-      <xdr:rowOff>111600</xdr:rowOff>
+      <xdr:rowOff>111240</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2354,7 +2392,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="0" y="2655720"/>
-        <a:ext cx="5759640" cy="3239640"/>
+        <a:ext cx="5759280" cy="3239280"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -4188,7 +4226,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="149.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="n">
         <v>25</v>
       </c>

</xml_diff>